<commit_message>
Update Bob inventory and disable unavailable weapon attacks
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R088c386a266b495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="Rd4b21403de7b4145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R911a7799db2647bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="Rfcb7bca2cb40473a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R5f6a7583897040b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="Rd24ad15df7a14624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R515385797db54ef7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R8543f4c9fbf6424d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,7 +212,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R840b80345aa54fcd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6bf2eaddf44e456e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1461,7 +1461,8 @@
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="5" t="str">
-        <x:v>Greatsword</x:v>
+        <x:f>IF(Inventory!B8&gt;0,"Greatsword","Greatsword (lost)")</x:f>
+        <x:v>Greatsword (lost)</x:v>
       </x:c>
       <x:c r="B48" s="11" t="n">
         <x:f>C18+E10</x:f>
@@ -1479,7 +1480,8 @@
       </x:c>
       <x:c r="F48" s="5"/>
       <x:c r="G48" s="5" t="str">
-        <x:v>Greatsword: two-handed, heavy. Great Weapon Fighting (see Journal).</x:v>
+        <x:f>IF(Inventory!B8&gt;0,"Greatsword: two-handed, heavy. Great Weapon Fighting (see Journal).","Greatsword lost: attack unavailable until recovered or replaced.")</x:f>
+        <x:v>Greatsword lost: attack unavailable until recovered or replaced.</x:v>
       </x:c>
       <x:c r="H48" s="5"/>
       <x:c r="I48" s="5"/>
@@ -1506,7 +1508,8 @@
       </x:c>
       <x:c r="F49" s="5"/>
       <x:c r="G49" s="5" t="str">
-        <x:v>Javelin: range 30/120 ft.</x:v>
+        <x:f>"Javelins carried: "&amp;Inventory!B9&amp;". Range 30/120 ft."</x:f>
+        <x:v>Javelins carried: 4. Range 30/120 ft.</x:v>
       </x:c>
       <x:c r="H49" s="5"/>
       <x:c r="I49" s="5"/>
@@ -1596,7 +1599,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9da48e2ada954e75"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75ed59d7c1914621"/>
 </x:worksheet>
 </file>
 
@@ -2828,7 +2831,7 @@
       </x:c>
       <x:c r="E4" s="24" t="n">
         <x:f>SUM(D8:D26)</x:f>
-        <x:v>77</x:v>
+        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
@@ -2869,17 +2872,17 @@
         <x:v>Greatsword</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C8" s="22" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="23" t="n">
         <x:f>IF(A8="","",B8*C8)</x:f>
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>Two-handed · heavy · 2d6 slashing</x:v>
+        <x:v>Lost; not carried. Two-handed, heavy; 2d6 slashing.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -2887,14 +2890,14 @@
         <x:v>Javelin</x:v>
       </x:c>
       <x:c r="B9" s="18" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C9" s="22" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D9" s="23" t="n">
         <x:f>IF(A9="","",B9*C9)</x:f>
-        <x:v>10</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
         <x:v>Thrown · range 30/120 ft · 1d6 piercing</x:v>
@@ -3236,16 +3239,17 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="260" customHeight="1">
+    <x:row r="13" ht="300" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
         <x:v>Imported from the June 17, 2026 character sheet and Greatsword Bob conversation. Uses the 2014 fifth-edition Paladin rules.
 DM CHECK — The paper sheet lists 120 gp alongside starting gear. Rolled starting gold normally replaces starting equipment; confirm which method your table uses. Do not automatically add the Noble’s 25 gp.
-Second martial weapon: not confirmed. Greatsword is confirmed.
+Second martial weapon: not confirmed. Greatsword was confirmed in the starting equipment; now lost.
 Fire resistance: halve fire damage. Position of Privilege: Noble background feature.
-Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.</x:v>
+Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.
+Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">

</xml_diff>

<commit_message>
Add detailed 2014 spell restrictions and compact spellbook layout
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R5f6a7583897040b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="Rd24ad15df7a14624"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R515385797db54ef7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R8543f4c9fbf6424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R736c6c57be674f17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R019448ec4bac4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R52cd4e9f58d64efe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R928faca91c79426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="Rdaf17f7e3f334059"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +22,7 @@
     <x:numFmt numFmtId="201" formatCode="+0;-0;0"/>
     <x:numFmt numFmtId="202" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -60,8 +61,25 @@
       <x:color rgb="FF182F43"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243347"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF243347"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,6 +106,26 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF183346"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDFE7EB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F1E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -100,7 +138,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -175,6 +213,43 @@
     <x:xf numFmtId="200" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -212,7 +287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6bf2eaddf44e456e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R06c5a06d36d34520"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1599,7 +1674,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75ed59d7c1914621"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8e19fa9de94251"/>
 </x:worksheet>
 </file>
 
@@ -1867,7 +1942,7 @@
         <x:v>Description</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="50" customHeight="1">
+    <x:row r="15" ht="66" customHeight="1">
       <x:c r="A15" s="18" t="str">
         <x:v>Command</x:v>
       </x:c>
@@ -1890,10 +1965,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
-        <x:v>Give a one-word command. A target that understands it makes a Wisdom save; restrictions apply.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="90" customHeight="1">
+        <x:v>One visible creature within 60 ft makes a Wisdom save. One-word command takes effect next turn. No effect on undead, a creature that cannot understand your language, or a directly harmful command. See Spell details for every command, targeting restrictions, and higher slots.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="66" customHeight="1">
       <x:c r="A16" s="18" t="str">
         <x:v>Purify Food and Drink</x:v>
       </x:c>
@@ -1916,10 +1991,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
-        <x:v>All nonmagical food and drink within a 5-foot-radius sphere centered on a point within range is purified and rendered free of poison and disease. Components: V, S. Ritual tag; the 2014 Paladin class does not grant ritual casting.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="50" customHeight="1">
+        <x:v>Purifies nonmagical food and drink in a 5-ft-radius sphere centered within 10 ft. Removes poison and disease only. V, S; no concentration. Bob cannot cast it as a ritual without a separate feature. Full limits are in Spell details.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="66" customHeight="1">
       <x:c r="A17" s="18" t="str">
         <x:v>Bless</x:v>
       </x:c>
@@ -1933,7 +2008,7 @@
         <x:v>30 ft</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>1 minute</x:v>
+        <x:v>Up to 1 minute</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
         <x:v>Yes</x:v>
@@ -1942,7 +2017,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
-        <x:v>Up to three creatures add 1d4 to attack rolls and saving throws. Higher slots add targets.</x:v>
+        <x:v>Up to 3 creatures within 30 ft, including Bob, add 1d4 to attack rolls and saves. V, S, M; concentration up to 1 minute. No bonus to damage or ability checks. Full components, concentration checks, and target restrictions are in Spell details.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
@@ -3280,9 +3355,13 @@
         <x:v>When you hit with a melee weapon attack, you may expend a 1st-level spell slot to deal 2d8 extra radiant damage, or 3d8 against an undead or fiend. Decide after the hit. Uses the same two spell slots as your prepared spells; slots return on a long rest. Great Weapon Fighting rerolls only the weapon damage dice, not Divine Smite dice.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="38" customHeight="1">
-      <x:c r="A18" s="18"/>
-      <x:c r="B18" s="18"/>
+    <x:row r="18" ht="44" customHeight="1">
+      <x:c r="A18" s="18" t="str">
+        <x:v>Spellcasting rules — 2014</x:v>
+      </x:c>
+      <x:c r="B18" s="18" t="str">
+        <x:v>Full casting restrictions, preparation, slots, armor, components, targeting, concentration, and sources are in the Spell details tab.</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="5"/>
@@ -3337,4 +3416,381 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="112" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="30" t="str">
+        <x:v>Bob’s detailed spell reference (2014)</x:v>
+      </x:c>
+      <x:c r="B1" s="30"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="28" t="str">
+        <x:v>Three prepared spells share two 1st-level slots. Divine Smite uses the same pool. Restore slots on a long rest.</x:v>
+      </x:c>
+      <x:c r="B2" s="28"/>
+    </x:row>
+    <x:row r="3" ht="23" customHeight="1">
+      <x:c r="A3" s="32" t="str">
+        <x:v>Rule / restriction</x:v>
+      </x:c>
+      <x:c r="B3" s="32" t="str">
+        <x:v>Details</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="33" t="str">
+        <x:v>Command</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>Level 1; 1 action; 60 ft; 1 round; no concentration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>School &amp; components</x:v>
+      </x:c>
+      <x:c r="B5" s="36" t="str">
+        <x:v>1st-level enchantment. Verbal (V) only: you must be able to speak the magic words. No somatic gesture, material, or focus is required. Not a ritual. No concentration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A6" s="37" t="str">
+        <x:v>Target &amp; save</x:v>
+      </x:c>
+      <x:c r="B6" s="38" t="str">
+        <x:v>Choose one creature you can see within 60 ft, with a clear path to it (no total cover). Speak a one-word command in a language it understands. The target makes a Wisdom saving throw against your spell save DC. On success, nothing happens; on failure, it follows the command on its next turn. You do not make a spell attack roll.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>No-effect restrictions</x:v>
+      </x:c>
+      <x:c r="B7" s="36" t="str">
+        <x:v>Undead are unaffected. The spell also has no effect if the target does not understand your language or the command would directly harm it. If it cannot follow the command, the spell ends. It does not grant ongoing control, extra commands, or a multi-step instruction. A failed effect or successful save does not refund your slot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="37" t="str">
+        <x:v>Approach</x:v>
+      </x:c>
+      <x:c r="B8" s="38" t="str">
+        <x:v>The target takes the shortest, most direct route toward you. If it gets within 5 ft of you, it ends its turn.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>Drop</x:v>
+      </x:c>
+      <x:c r="B9" s="36" t="str">
+        <x:v>The target drops what it is holding, then ends its turn. This does not automatically remove worn armor or other worn equipment.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="37" t="str">
+        <x:v>Flee</x:v>
+      </x:c>
+      <x:c r="B10" s="38" t="str">
+        <x:v>The target spends its turn moving away from you by the fastest means it has available.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="35" t="str">
+        <x:v>Grovel</x:v>
+      </x:c>
+      <x:c r="B11" s="36" t="str">
+        <x:v>The target falls prone, then ends its turn. Prone means its attacks have disadvantage; attacks against it have advantage within 5 ft and disadvantage from farther away. Standing later costs half its speed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A12" s="37" t="str">
+        <x:v>Halt</x:v>
+      </x:c>
+      <x:c r="B12" s="38" t="str">
+        <x:v>The target stays in place and takes no actions. A flying target remains aloft if it can; if it must keep moving to stay airborne, it moves only the minimum necessary.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A13" s="35" t="str">
+        <x:v>Other words &amp; rulings</x:v>
+      </x:c>
+      <x:c r="B13" s="36" t="str">
+        <x:v>Other one-word commands are allowed, but the DM decides how the target responds and what counts as directly harmful. The spell does not impose the charmed condition, so immunity to being charmed alone is not a stated exclusion; other creature traits can still affect the saving throw or magic.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="37" t="str">
+        <x:v>Higher slots</x:v>
+      </x:c>
+      <x:c r="B14" s="38" t="str">
+        <x:v>A slot of 2nd level or higher adds one target per slot level above 1st. Each target must meet the normal requirements and make its own save. All chosen targets must be within 30 ft of one another when selected. Bob has no higher-level slots at level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="35" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B15" s="36" t="str">
+        <x:v>https://www.dnd5eapi.co/api/2014/spells/command</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="33" t="str">
+        <x:v>Purify Food and Drink</x:v>
+      </x:c>
+      <x:c r="B16" s="33" t="str">
+        <x:v>Level 1; 1 action; 10 ft; Instantaneous; no concentration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A17" s="35" t="str">
+        <x:v>School &amp; components</x:v>
+      </x:c>
+      <x:c r="B17" s="36" t="str">
+        <x:v>1st-level transmutation. Verbal and somatic (V, S): you must be able to speak and have free use of at least one hand. No material or focus is required. No concentration. No saving throw or spell attack roll.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A18" s="37" t="str">
+        <x:v>Area &amp; effect</x:v>
+      </x:c>
+      <x:c r="B18" s="38" t="str">
+        <x:v>Choose a point within 10 ft. All nonmagical food and drink inside a 5-ft-radius sphere around that point becomes free of poison and disease. The 10-ft limit applies to the center; the sphere extends 5 ft from it in every direction, including the center itself.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A19" s="35" t="str">
+        <x:v>Targeting restrictions</x:v>
+      </x:c>
+      <x:c r="B19" s="36" t="str">
+        <x:v>You need a clear path to the point; total cover blocks targeting and blocks the area spreading through it. Seeing the point is not an explicit spell requirement. Whether a closed container blocks the magic depends on whether it provides total cover, so resolve that with the DM.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A20" s="37" t="str">
+        <x:v>What it does not do</x:v>
+      </x:c>
+      <x:c r="B20" s="38" t="str">
+        <x:v>It does not affect magical food or drink, cure a poisoned or diseased creature, create food or water, detect poison, or make every non-food substance edible. It only removes poison and disease from qualifying food and drink. Other contamination, spoilage, and whether something counts as food or drink may require a DM ruling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A21" s="35" t="str">
+        <x:v>Duration</x:v>
+      </x:c>
+      <x:c r="B21" s="36" t="str">
+        <x:v>The purification happens immediately. You do not maintain it, and dispelling magic afterward does not undo an instantaneous purification. The food or drink can be contaminated again later; it gains no lasting protective ward.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A22" s="37" t="str">
+        <x:v>Ritual restriction</x:v>
+      </x:c>
+      <x:c r="B22" s="38" t="str">
+        <x:v>The spell has a ritual tag, but the 2014 Paladin class does not grant ritual casting. Bob must prepare it and spend 1 spell slot for his normal 1-action cast. Only a separate feature that actually permits this spell as a ritual would allow a slot-free casting with 10 additional minutes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A23" s="35" t="str">
+        <x:v>Higher slots</x:v>
+      </x:c>
+      <x:c r="B23" s="36" t="str">
+        <x:v>You may spend a higher-level slot if available, but this spell lists no increase in radius, range, or effect. Bob has only 1st-level slots at level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="37" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B24" s="38" t="str">
+        <x:v>https://www.dnd5eapi.co/api/2014/spells/purify-food-and-drink</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="33" t="str">
+        <x:v>Bless</x:v>
+      </x:c>
+      <x:c r="B25" s="33" t="str">
+        <x:v>Level 1; 1 action; 30 ft; Up to 1 minute; concentration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A26" s="37" t="str">
+        <x:v>School &amp; components</x:v>
+      </x:c>
+      <x:c r="B26" s="38" t="str">
+        <x:v>1st-level enchantment. Verbal, somatic, and material (V, S, M): a sprinkling of holy water. This spell states no component cost and does not say the material is consumed. A component pouch or your Paladin holy-symbol focus can replace that material. You still need speech and the required hand access; the hand used for the material or focus can also perform the somatic gesture. Not a ritual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A27" s="35" t="str">
+        <x:v>Targets</x:v>
+      </x:c>
+      <x:c r="B27" s="36" t="str">
+        <x:v>Choose up to three creatures within 30 ft, including yourself if desired. You need a clear path to each target; total cover blocks targeting. The spell does not explicitly require sight or a willing target, and lists no creature-type exclusion. No saving throw or spell attack is required.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A28" s="37" t="str">
+        <x:v>Benefit</x:v>
+      </x:c>
+      <x:c r="B28" s="38" t="str">
+        <x:v>Until the spell ends, each target can roll 1d4 and add it whenever it makes an attack roll or saving throw. Roll the bonus for each eligible roll; it is not used up after one roll. This includes death saving throws. It does not add to damage, AC, ability checks, skill checks, or initiative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A29" s="35" t="str">
+        <x:v>Duration &amp; range</x:v>
+      </x:c>
+      <x:c r="B29" s="36" t="str">
+        <x:v>Concentration, up to 1 minute (normally 10 combat rounds). Once cast, targets can move beyond 30 ft without losing the spell. You cannot transfer the benefit to new targets without casting again. Multiple Bless castings on one target do not stack into extra d4s.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A30" s="37" t="str">
+        <x:v>Concentration limits</x:v>
+      </x:c>
+      <x:c r="B30" s="38" t="str">
+        <x:v>You may concentrate on only one spell at a time. Casting another concentration spell, being incapacitated, or dying ends Bless. You may end it voluntarily at any time without an action. Ordinary movement and attacks do not break it. Casting Command or Purify Food and Drink does not itself break Bless because neither requires concentration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A31" s="35" t="str">
+        <x:v>Damage checks</x:v>
+      </x:c>
+      <x:c r="B31" s="36" t="str">
+        <x:v>Each separate source of damage requires your Constitution saving throw: DC 10 or half the damage actually taken, whichever is higher (round fractions down). Failure ends Bless for every target. Your Constitution save bonus is shown in the casting reference below. If you included yourself in Bless, its d4 applies to this save while the spell is still active. The DM can also call for a DC 10 check for severe environmental disruption.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A32" s="37" t="str">
+        <x:v>Higher slots</x:v>
+      </x:c>
+      <x:c r="B32" s="38" t="str">
+        <x:v>Add one target for each slot level above 1st: four targets with a 2nd-level slot, five with a 3rd-level slot, and so on. Each starts within 30 ft of you; there is no additional distance-between-targets restriction. Higher slots do not increase the d4 or duration. Bob cannot upcast at level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="35" t="str">
+        <x:v>Source</x:v>
+      </x:c>
+      <x:c r="B33" s="36" t="str">
+        <x:v>https://www.dnd5eapi.co/api/2014/spells/bless</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="33" t="str">
+        <x:v>Shared casting rules</x:v>
+      </x:c>
+      <x:c r="B34" s="33" t="str">
+        <x:v>Applies to Bob’s 2014 Paladin spellcasting</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A35" s="35" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="B35" s="36" t="str">
+        <x:v>Your prepared-spell limit is Charisma modifier + half Paladin level rounded down, minimum 1 once spellcasting starts at level 2. Choose Paladin spells of levels for which you have slots. You can change the list after a long rest, with at least 1 minute of prayer and meditation per spell level for every spell on the new list. Bob's three 1st-level spells take at least 3 minutes to prepare. Casting a spell does not unprepare it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A36" s="37" t="str">
+        <x:v>Slots &amp; recovery</x:v>
+      </x:c>
+      <x:c r="B36" s="38" t="str">
+        <x:v>Every normal cast uses one slot of the spell's level or higher. Command, Purify Food and Drink, Bless, and Divine Smite share Bob's two 1st-level slots at level 2. Two uses total, in any combination. A long rest restores spent slots; a short rest does not. A target succeeding on its save or a spell ending early does not refund a spent slot.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A37" s="35" t="str">
+        <x:v>Actions &amp; armor</x:v>
+      </x:c>
+      <x:c r="B37" s="36" t="str">
+        <x:v>All three recorded spells take 1 action, so they normally use the action you could otherwise use to attack. Under 2014 rules, casting any bonus-action spell on your turn limits other spells that turn to a cantrip with a casting time of 1 action. This is not a blanket one-spell-per-turn rule. Bob can cast in his chain mail because he is proficient with it; wearing armor you lack proficiency in prevents spellcasting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A38" s="37" t="str">
+        <x:v>Speech &amp; hands</x:v>
+      </x:c>
+      <x:c r="B38" s="38" t="str">
+        <x:v>All three spells need verbal components, so being gagged or inside magical silence prevents their casting. Purify and Bless also require somatic gestures. A hand holding a weapon cannot freely perform those gestures unless another rule permits it. A focus can replace only eligible material components, not verbal or somatic requirements. Purify has no material component, so merely holding a focus does not remove its free-hand requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A39" s="35" t="str">
+        <x:v>Holy symbol</x:v>
+      </x:c>
+      <x:c r="B39" s="36" t="str">
+        <x:v>A Paladin can use a holy symbol as a spellcasting focus, holding it, wearing it visibly, or bearing it on a shield. Bob has a holy symbol recorded, but its form is unconfirmed. Bless's material can be replaced by this focus; a separately specified costly or consumed material would still have to be supplied. Neither Command nor Purify needs a material component.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A40" s="37" t="str">
+        <x:v>Choosing targets</x:v>
+      </x:c>
+      <x:c r="B40" s="38" t="str">
+        <x:v>At casting, obey the spell's range, target type, sight requirement if stated, and clear-path rule. Total cover blocks targeting, even when a target is visible through an obstruction. Effects normally continue beyond casting range unless the spell says otherwise. Areas spread from their origin in unblocked straight lines; total cover excludes the blocked part.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A41" s="35" t="str">
+        <x:v>Concentration</x:v>
+      </x:c>
+      <x:c r="B41" s="36" t="str">
+        <x:v>Only Bless among Bob's three spells needs it. Keep one concentration effect at a time. Damage checks use Constitution, not Charisma and not your spell save DC. Each damage source has its own check, DC max(10, half damage taken rounded down). Incapacitation, death, a new concentration spell, voluntary ending, or a failed required check ends it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A42" s="37" t="str">
+        <x:v>Saves versus attacks</x:v>
+      </x:c>
+      <x:c r="B42" s="38" t="str">
+        <x:v>Command makes its target roll Wisdom against your spell save DC. Bless and Purify require neither a save nor a spell attack roll. Your spell attack modifier therefore is not rolled for any of these three spells. Divine Smite is a class feature triggered by a melee weapon hit, not a separate spell attack; a thrown javelin does not qualify, but a melee javelin hit can.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="66" hidden="0" customHeight="1">
+      <x:c r="A43" s="35" t="str">
+        <x:v>Rules sources</x:v>
+      </x:c>
+      <x:c r="B43" s="36" t="str">
+        <x:v>2014 SRD 5.1 spell and spellcasting rules, paraphrased with practical notes. Sources: https://www.dnd5eapi.co/api/2014/rule-sections/casting-a-spell ; https://www.dnd5eapi.co/api/2014/rule-sections/what-is-a-spell ; https://www.dnd5eapi.co/api/2014/classes/paladin . Source text: https://media.wizards.com/2023/downloads/dnd/SRD_CC_v5.1.pdf . SRD 5.1 by Wizards of the Coast LLC is licensed under CC BY 4.0: https://creativecommons.org/licenses/by/4.0/ . Specific creature traits and your DM's rulings can change an interaction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="28"/>
+      <x:c r="B44" s="28"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="28"/>
+      <x:c r="B45" s="28"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="28"/>
+      <x:c r="B46" s="28"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="28"/>
+      <x:c r="B47" s="28"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="28"/>
+      <x:c r="B48" s="28"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:B1"/>
+    <x:mergeCell ref="A2:B2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Bob's Bless cast and encounter notes
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R736c6c57be674f17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R019448ec4bac4669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R52cd4e9f58d64efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R928faca91c79426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="Rdaf17f7e3f334059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Ra586e6edf63a42c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R5eafa9616c9e445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R56954585ff2f4712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R38edc5aef51948b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R12e3a95fa7d3457f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -287,7 +287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R06c5a06d36d34520"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R491b37859533404c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1674,7 +1674,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad8e19fa9de94251"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0830c1f288649a3"/>
 </x:worksheet>
 </file>
 
@@ -1779,11 +1779,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="9" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
         <x:f>B7-C7</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5" t="str">
@@ -3314,7 +3314,7 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="300" customHeight="1">
+    <x:row r="13" ht="380" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
@@ -3324,7 +3324,8 @@
 Second martial weapon: not confirmed. Greatsword was confirmed in the starting equipment; now lost.
 Fire resistance: halve fire damage. Position of Privilege: Noble background feature.
 Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.
-Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.</x:v>
+Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.
+Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">

</xml_diff>

<commit_message>
Update Bob to 13 HP after falling rocks
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Ra586e6edf63a42c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R5eafa9616c9e445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R56954585ff2f4712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R38edc5aef51948b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R12e3a95fa7d3457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R3300027ab0ff4a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R51bbc7ea7518405a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="Rcc4797d50cf04bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R3e7aa71196c44bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="Rd17f21ec094545fb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -287,7 +287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R491b37859533404c"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7020972dbed44415"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -917,7 +917,7 @@
         <x:v>Current HP</x:v>
       </x:c>
       <x:c r="H22" s="9" t="n">
-        <x:v>15</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="I22" s="5"/>
       <x:c r="J22" s="5"/>
@@ -1674,7 +1674,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0830c1f288649a3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R175cbee66c084f62"/>
 </x:worksheet>
 </file>
 
@@ -3314,7 +3314,7 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="380" customHeight="1">
+    <x:row r="13" ht="440" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
@@ -3325,7 +3325,8 @@
 Fire resistance: halve fire damage. Position of Privilege: Noble background feature.
 Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.
 Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.
-Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.</x:v>
+Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.
+Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Bless concentration save required: Constitution d20 + 1 against DC 10. Result pending; continued Bless on the druid, Cat, and Taric is not yet confirmed. Bob is not a Bless target and does not add its d4 to this save. One 1st-level spell slot remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">

</xml_diff>

<commit_message>
Clear obsolete Bless concentration save reminder
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R3300027ab0ff4a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R51bbc7ea7518405a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="Rcc4797d50cf04bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R3e7aa71196c44bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="Rd17f21ec094545fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Ra2309474d49f427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R8794f4bf67c84041"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R4742a8179db34312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="Ra1d602c1486c490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R09e53934dee14de3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -287,7 +287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7020972dbed44415"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb53d2a8fbc974f83"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1674,7 +1674,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R175cbee66c084f62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78adf1b1059476b"/>
 </x:worksheet>
 </file>
 
@@ -3326,7 +3326,7 @@
 Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.
 Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.
 Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.
-Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Bless concentration save required: Constitution d20 + 1 against DC 10. Result pending; continued Bless on the druid, Cat, and Taric is not yet confirmed. Bob is not a Bless target and does not add its d4 to this save. One 1st-level spell slot remains.</x:v>
+Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Kai clarified that Bless had already ended. The druid, Cat, and Taric no longer receive its bonus; no concentration save was needed for this damage. One 1st-level spell slot remains.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">

</xml_diff>

<commit_message>
Show covered condition and temporary Charisma penalty
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Ra2309474d49f427c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R8794f4bf67c84041"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R4742a8179db34312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="Ra1d602c1486c490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R09e53934dee14de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Rc78a0d92a12b4651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R4ba34c3cdd3c4ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R269e8aa7b6d249e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R53e7b3363fd244ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R95c00742d9c84f24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -287,7 +287,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb53d2a8fbc974f83"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc8813b8a2a454899"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -928,18 +928,18 @@
         <x:v>CHA</x:v>
       </x:c>
       <x:c r="B23" s="9" t="n">
-        <x:v>14</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C23" s="11" t="n">
         <x:f>INT((B23-10)/2)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E23" s="11" t="n">
         <x:f>C23+IF(D23="Yes",$E$10,0)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F23" s="5"/>
       <x:c r="G23" s="5" t="str">
@@ -1131,7 +1131,7 @@
       </x:c>
       <x:c r="D31" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B31,$A$18:$A$23,0))+IF(C31="Yes",$E$10,0)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="5"/>
       <x:c r="F31" s="5"/>
@@ -1207,7 +1207,7 @@
       </x:c>
       <x:c r="D34" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B34,$A$18:$A$23,0))+IF(C34="Yes",$E$10,0)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E34" s="5"/>
       <x:c r="F34" s="5"/>
@@ -1357,7 +1357,7 @@
       </x:c>
       <x:c r="D39" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B39,$A$18:$A$23,0))+IF(C39="Yes",$E$10,0)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E39" s="5"/>
       <x:c r="F39" s="5"/>
@@ -1379,7 +1379,7 @@
       </x:c>
       <x:c r="D40" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B40,$A$18:$A$23,0))+IF(C40="Yes",$E$10,0)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E40" s="5"/>
       <x:c r="F40" s="5"/>
@@ -1674,7 +1674,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra78adf1b1059476b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a67b1e770214f27"/>
 </x:worksheet>
 </file>
 
@@ -1766,7 +1766,7 @@
       </x:c>
       <x:c r="G6" s="10" t="n">
         <x:f>IF(Character!B10&lt;2,"Not unlocked",8+Character!E10+Character!C23)</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H6" s="5"/>
     </x:row>
@@ -1791,7 +1791,7 @@
       </x:c>
       <x:c r="G7" s="11" t="n">
         <x:f>IF(Character!B10&lt;2,"Not unlocked",Character!E10+Character!C23)</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H7" s="5"/>
     </x:row>
@@ -1816,7 +1816,7 @@
       </x:c>
       <x:c r="G8" s="10" t="n">
         <x:f>IF(Character!B10&lt;2,0,MAX(1,Character!C23+INT(Character!B10/2)))</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H8" s="5"/>
     </x:row>
@@ -1866,7 +1866,7 @@
       </x:c>
       <x:c r="G10" s="10" t="str">
         <x:f>IF(G9&gt;G8,"Over limit","Within limit")</x:f>
-        <x:v>Within limit</x:v>
+        <x:v>Over limit</x:v>
       </x:c>
       <x:c r="H10" s="5"/>
     </x:row>
@@ -3314,7 +3314,7 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="440" customHeight="1">
+    <x:row r="13" ht="500" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
@@ -3326,7 +3326,8 @@
 Resource counters start full because spent uses were not recorded. XP is set to 0 as a starting placeholder. Equipment weights of 0 mean not recorded, not weightless.
 Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.
 Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.
-Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Kai clarified that Bless had already ended. The druid, Cat, and Taric no longer receive its bonus; no concentration save was needed for this damage. One 1st-level spell slot remains.</x:v>
+Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Kai clarified that Bless had already ended. The druid, Cat, and Taric no longer receive its bonus; no concentration save was needed for this damage. One 1st-level spell slot remains.
+Covered in blood and guts — September 13, 2026 (Kai): -2 Charisma until Bob takes a bath. Applied to the score: 14 to 12, modifier +1. Base score 14 is retained here for restoration after bathing. HP stays 13/20 and one 1st-level spell slot remains. The three prepared spells are retained; the reduced preparation limit of 2 needs a DM ruling. Divine Sense counters are unchanged pending the DM ruling on how this temporary effect affects its pool.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
@@ -3365,9 +3366,13 @@
         <x:v>Full casting restrictions, preparation, slots, armor, components, targeting, concentration, and sources are in the Spell details tab.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="5"/>
-      <x:c r="B19" s="5"/>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="17" t="str">
+        <x:v>Covered in blood and guts</x:v>
+      </x:c>
+      <x:c r="B19" s="17" t="str">
+        <x:v>Temporary -2 Charisma score until Bob takes a bath: base 14, current 12 (+1 modifier). Restore Charisma to 14 after the bath. Spell save DC 11; spell attack +3; Charisma save +3. Current prepared-spell limit is 2; all 3 already-prepared spells are retained pending the DM ruling on this temporary penalty.</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="19" t="str">

</xml_diff>

<commit_message>
Update Bob spell selection and detailed casting reference
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="Rc78a0d92a12b4651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R4ba34c3cdd3c4ad4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R269e8aa7b6d249e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R53e7b3363fd244ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R95c00742d9c84f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R76a66233b52d44c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="Rcceadbd1eb0f4cc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="Rb457a6852da84252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R52359aa56af64ce9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R8bbb0fb33a87437c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="13">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -126,6 +126,21 @@
         <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF183346"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F1E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -138,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="45">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -248,6 +263,24 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -287,7 +320,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc8813b8a2a454899"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8cbf8847dd894e5f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1674,7 +1707,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a67b1e770214f27"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e4a86900c94d28"/>
 </x:worksheet>
 </file>
 
@@ -1944,7 +1977,7 @@
     </x:row>
     <x:row r="15" ht="66" customHeight="1">
       <x:c r="A15" s="18" t="str">
-        <x:v>Command</x:v>
+        <x:v>Cure Wounds</x:v>
       </x:c>
       <x:c r="B15" s="18" t="n">
         <x:v>1</x:v>
@@ -1953,10 +1986,10 @@
         <x:v>1 action</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
-        <x:v>60 ft</x:v>
+        <x:v>Touch</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>1 round</x:v>
+        <x:v>Instantaneous</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
         <x:v>No</x:v>
@@ -1965,12 +1998,12 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
-        <x:v>One visible creature within 60 ft makes a Wisdom save. One-word command takes effect next turn. No effect on undead, a creature that cannot understand your language, or a directly harmful command. See Spell details for every command, targeting restrictions, and higher slots.</x:v>
+        <x:v>Touch one creature to heal 1d8 + Charisma modifier HP. V, S; no concentration. No effect on undead or constructs. Cannot exceed maximum HP or revive the dead. Full rules in Spell details.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="66" customHeight="1">
       <x:c r="A16" s="18" t="str">
-        <x:v>Purify Food and Drink</x:v>
+        <x:v>Heroism</x:v>
       </x:c>
       <x:c r="B16" s="18" t="n">
         <x:v>1</x:v>
@@ -1979,33 +2012,33 @@
         <x:v>1 action</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
-        <x:v>10 ft</x:v>
+        <x:v>Touch</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>Instantaneous</x:v>
+        <x:v>Up to 1 minute</x:v>
       </x:c>
       <x:c r="F16" s="18" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="G16" s="18" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
-        <x:v>Purifies nonmagical food and drink in a 5-ft-radius sphere centered within 10 ft. Removes poison and disease only. V, S; no concentration. Bob cannot cast it as a ritual without a separate feature. Full limits are in Spell details.</x:v>
+        <x:v>Touch one willing creature, including yourself or a party member: immune to frightened; temporary HP equal to Charisma modifier at the start of each target turn. V, S; concentration. Temporary HP do not stack and vanish when the spell ends. Full rules in Spell details.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="66" customHeight="1">
       <x:c r="A17" s="18" t="str">
-        <x:v>Bless</x:v>
+        <x:v>Thunderous Smite</x:v>
       </x:c>
       <x:c r="B17" s="18" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
-        <x:v>1 action</x:v>
+        <x:v>1 bonus action</x:v>
       </x:c>
       <x:c r="D17" s="18" t="str">
-        <x:v>30 ft</x:v>
+        <x:v>Self</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
         <x:v>Up to 1 minute</x:v>
@@ -2017,7 +2050,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
-        <x:v>Up to 3 creatures within 30 ft, including Bob, add 1d4 to attack rolls and saves. V, S, M; concentration up to 1 minute. No bonus to damage or ability checks. Full components, concentration checks, and target restrictions are in Spell details.</x:v>
+        <x:v>Cast before a melee weapon hit: first hit adds 2d6 thunder; creature makes Strength save vs spell DC or is pushed 10 ft and knocked prone. V only; concentration; audible 300 ft. Melee javelin qualifies; thrown does not. Full rules in Spell details.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
@@ -3314,7 +3347,7 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="500" customHeight="1">
+    <x:row r="13" ht="570" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
@@ -3327,7 +3360,8 @@
 Inventory update — September 13, 2026: greatsword lost (0 carried); javelins reduced from 5 to 4, per Kai.
 Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.
 Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Kai clarified that Bless had already ended. The druid, Cat, and Taric no longer receive its bonus; no concentration save was needed for this damage. One 1st-level spell slot remains.
-Covered in blood and guts — September 13, 2026 (Kai): -2 Charisma until Bob takes a bath. Applied to the score: 14 to 12, modifier +1. Base score 14 is retained here for restoration after bathing. HP stays 13/20 and one 1st-level spell slot remains. The three prepared spells are retained; the reduced preparation limit of 2 needs a DM ruling. Divine Sense counters are unchanged pending the DM ruling on how this temporary effect affects its pool.</x:v>
+Covered in blood and guts — September 13, 2026 (Kai): -2 Charisma until Bob takes a bath. Applied to the score: 14 to 12, modifier +1. Base score 14 is retained here for restoration after bathing. HP stays 13/20 and one 1st-level spell slot remains. The three prepared spells are retained; the reduced preparation limit of 2 needs a DM ruling. Divine Sense counters are unchanged pending the DM ruling on how this temporary effect affects its pool.
+Spell selection — September 14, 2026 (Kai): Cure Wounds, Heroism, and Thunderous Smite replace Command, Purify Food and Drink, and Bless in the recorded list. This records the requested next preparation; no completed long rest, bath, healing, casting, or resource recovery is assumed. HP remains 13/20; one 1st-level slot remains. The current preparation limit is 2 with Charisma 12; all three choices are retained pending bathing (restoring Charisma 14 and limit 3) or the DM’s ruling. Heroism and Thunderous Smite cannot be concentrated on together.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
@@ -3371,7 +3405,7 @@
         <x:v>Covered in blood and guts</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>Temporary -2 Charisma score until Bob takes a bath: base 14, current 12 (+1 modifier). Restore Charisma to 14 after the bath. Spell save DC 11; spell attack +3; Charisma save +3. Current prepared-spell limit is 2; all 3 already-prepared spells are retained pending the DM ruling on this temporary penalty.</x:v>
+        <x:v>Temporary -2 Charisma score until Bob takes a bath: base 14, current 12 (+1 modifier). Restore Charisma to 14 after the bath. Spell save DC 11; spell attack +3; Charisma save +3. Current prepared-spell limit is 2; all 3 selected spells are recorded pending the DM ruling on this temporary penalty.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
@@ -3439,9 +3473,9 @@
       </x:c>
       <x:c r="B1" s="30"/>
     </x:row>
-    <x:row r="2" ht="30" customHeight="1">
+    <x:row r="2" ht="44" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>Three prepared spells share two 1st-level slots. Divine Smite uses the same pool. Restore slots on a long rest.</x:v>
+        <x:v>3 selections recorded; current preparation limit 2 (DM check). Two shared 1st-level slots; 1 remains. Heroism and Thunderous Smite cannot be maintained together. No rest or bath assumed.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
     </x:row>
@@ -3454,324 +3488,316 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="33" t="str">
-        <x:v>Command</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="str">
-        <x:v>Level 1; 1 action; 60 ft; 1 round; no concentration</x:v>
+      <x:c r="A4" s="40" t="str">
+        <x:v>Cure Wounds</x:v>
+      </x:c>
+      <x:c r="B4" s="40" t="str">
+        <x:v>Level 1; 1 action; Touch; Instantaneous; no concentration</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A5" s="35" t="str">
+      <x:c r="A5" s="41" t="str">
         <x:v>School &amp; components</x:v>
       </x:c>
-      <x:c r="B5" s="36" t="str">
-        <x:v>1st-level enchantment. Verbal (V) only: you must be able to speak the magic words. No somatic gesture, material, or focus is required. Not a ritual. No concentration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A6" s="37" t="str">
-        <x:v>Target &amp; save</x:v>
-      </x:c>
-      <x:c r="B6" s="38" t="str">
-        <x:v>Choose one creature you can see within 60 ft, with a clear path to it (no total cover). Speak a one-word command in a language it understands. The target makes a Wisdom saving throw against your spell save DC. On success, nothing happens; on failure, it follows the command on its next turn. You do not make a spell attack roll.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A7" s="35" t="str">
-        <x:v>No-effect restrictions</x:v>
-      </x:c>
-      <x:c r="B7" s="36" t="str">
-        <x:v>Undead are unaffected. The spell also has no effect if the target does not understand your language or the command would directly harm it. If it cannot follow the command, the spell ends. It does not grant ongoing control, extra commands, or a multi-step instruction. A failed effect or successful save does not refund your slot.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="37" t="str">
-        <x:v>Approach</x:v>
-      </x:c>
-      <x:c r="B8" s="38" t="str">
-        <x:v>The target takes the shortest, most direct route toward you. If it gets within 5 ft of you, it ends its turn.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="35" t="str">
-        <x:v>Drop</x:v>
-      </x:c>
-      <x:c r="B9" s="36" t="str">
-        <x:v>The target drops what it is holding, then ends its turn. This does not automatically remove worn armor or other worn equipment.</x:v>
+      <x:c r="B5" s="42" t="str">
+        <x:v>1st-level evocation (2014). Verbal and somatic (V, S): speak and use at least one free hand for gestures. No material component or holy symbol is required. Not a ritual; no concentration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" s="43" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="str">
+        <x:v>Touch one creature, including yourself or a party member. Party members count as creatures. No attack roll, saving throw, or willing-target requirement is stated. You must be able to reach and touch the target; total cover blocks targeting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>Healing</x:v>
+      </x:c>
+      <x:c r="B7" s="42" t="str">
+        <x:v>Restore 1d8 + your Charisma modifier hit points with a 1st-level slot. Healing cannot exceed the target’s maximum HP and does not grant temporary HP. Use your current modifier shown above; this is the 2014 version, not the 2024 2d8 version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="43" t="str">
+        <x:v>Restrictions</x:v>
+      </x:c>
+      <x:c r="B8" s="44" t="str">
+        <x:v>No effect on undead or constructs. Does not revive a dead creature, regrow body parts, remove poison or disease, or automatically remove other conditions. A living creature at 0 HP regains consciousness when healing raises it above 0, unless another effect keeps it unconscious; its death-save successes and failures reset.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A9" s="41" t="str">
+        <x:v>Timing &amp; duration</x:v>
+      </x:c>
+      <x:c r="B9" s="42" t="str">
+        <x:v>The healing happens immediately and does not require ongoing concentration. Casting it does not itself end Heroism or Thunderous Smite. You cannot cast it on a turn when you cast a bonus-action spell under 2014 rules.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="37" t="str">
-        <x:v>Flee</x:v>
-      </x:c>
-      <x:c r="B10" s="38" t="str">
-        <x:v>The target spends its turn moving away from you by the fastest means it has available.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="35" t="str">
-        <x:v>Grovel</x:v>
-      </x:c>
-      <x:c r="B11" s="36" t="str">
-        <x:v>The target falls prone, then ends its turn. Prone means its attacks have disadvantage; attacks against it have advantage within 5 ft and disadvantage from farther away. Standing later costs half its speed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A12" s="37" t="str">
-        <x:v>Halt</x:v>
-      </x:c>
-      <x:c r="B12" s="38" t="str">
-        <x:v>The target stays in place and takes no actions. A flying target remains aloft if it can; if it must keep moving to stay airborne, it moves only the minimum necessary.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A13" s="35" t="str">
-        <x:v>Other words &amp; rulings</x:v>
-      </x:c>
-      <x:c r="B13" s="36" t="str">
-        <x:v>Other one-word commands are allowed, but the DM decides how the target responds and what counts as directly harmful. The spell does not impose the charmed condition, so immunity to being charmed alone is not a stated exclusion; other creature traits can still affect the saving throw or magic.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A14" s="37" t="str">
+      <x:c r="A10" s="43" t="str">
         <x:v>Higher slots</x:v>
       </x:c>
-      <x:c r="B14" s="38" t="str">
-        <x:v>A slot of 2nd level or higher adds one target per slot level above 1st. Each target must meet the normal requirements and make its own save. All chosen targets must be within 30 ft of one another when selected. Bob has no higher-level slots at level 2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="35" t="str">
+      <x:c r="B10" s="44" t="str">
+        <x:v>Add 1d8 healing for each slot level above 1st; add your Charisma modifier only once. Bob has only 1st-level slots at Paladin level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="41" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="B15" s="36" t="str">
-        <x:v>https://www.dnd5eapi.co/api/2014/spells/command</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="33" t="str">
-        <x:v>Purify Food and Drink</x:v>
-      </x:c>
-      <x:c r="B16" s="33" t="str">
-        <x:v>Level 1; 1 action; 10 ft; Instantaneous; no concentration</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A17" s="35" t="str">
+      <x:c r="B11" s="42" t="str">
+        <x:v>https://www.dnd5eapi.co/api/2014/spells/cure-wounds</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="40" t="str">
+        <x:v>Heroism</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str">
+        <x:v>Level 1; 1 action; Touch; Up to 1 minute; concentration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="41" t="str">
         <x:v>School &amp; components</x:v>
       </x:c>
-      <x:c r="B17" s="36" t="str">
-        <x:v>1st-level transmutation. Verbal and somatic (V, S): you must be able to speak and have free use of at least one hand. No material or focus is required. No concentration. No saving throw or spell attack roll.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A18" s="37" t="str">
-        <x:v>Area &amp; effect</x:v>
-      </x:c>
-      <x:c r="B18" s="38" t="str">
-        <x:v>Choose a point within 10 ft. All nonmagical food and drink inside a 5-ft-radius sphere around that point becomes free of poison and disease. The 10-ft limit applies to the center; the sphere extends 5 ft from it in every direction, including the center itself.</x:v>
+      <x:c r="B13" s="42" t="str">
+        <x:v>1st-level enchantment (2014). Verbal and somatic (V, S): speech and a free hand for gestures. No material or focus required. Not a ritual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A14" s="43" t="str">
+        <x:v>Target</x:v>
+      </x:c>
+      <x:c r="B14" s="44" t="str">
+        <x:v>Touch one willing creature, including a willing party member or yourself. Party members count as creatures. No creature-type exclusion, attack roll, or saving throw is stated. You need a clear path and must touch the target when casting; afterward it can move away. You cannot transfer the spell to someone else without another cast.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A15" s="41" t="str">
+        <x:v>Benefits &amp; timing</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="str">
+        <x:v>The target is immune to being frightened for the duration. At the start of each of that target’s turns, it gains temporary HP equal to your Charisma modifier. This is not immediate healing on casting and is not triggered at the start of Bob’s turn unless Bob is the target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A16" s="43" t="str">
+        <x:v>Temporary HP restrictions</x:v>
+      </x:c>
+      <x:c r="B16" s="44" t="str">
+        <x:v>Temporary HP do not stack or add up each round. When offered another pool, choose the existing pool or the new one. They absorb damage before normal HP and can coexist with full normal HP, but do not restore normal HP, wake a creature at 0 HP, or stabilize it. Damage absorbed by temporary HP still triggers a concentration save for the concentrating creature.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A17" s="41" t="str">
+        <x:v>Duration &amp; ending</x:v>
+      </x:c>
+      <x:c r="B17" s="42" t="str">
+        <x:v>Concentration up to 1 minute, normally 10 rounds. When Heroism ends, its frightened immunity and any remaining temporary HP from this spell end. It does not remove an underlying fear effect permanently; that effect can apply again if still active. Temporary HP from another source are not removed by Heroism ending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A18" s="43" t="str">
+        <x:v>Concentration conflict</x:v>
+      </x:c>
+      <x:c r="B18" s="44" t="str">
+        <x:v>Casting Thunderous Smite or any other concentration spell ends your Heroism. Damage to Bob requires a Constitution concentration save, even if the protected target is someone else. Damage to another target does not itself make Bob save. Ordinary attacks, movement, and casting Cure Wounds do not themselves break concentration. See shared rules for all ending conditions.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A19" s="35" t="str">
-        <x:v>Targeting restrictions</x:v>
-      </x:c>
-      <x:c r="B19" s="36" t="str">
-        <x:v>You need a clear path to the point; total cover blocks targeting and blocks the area spreading through it. Seeing the point is not an explicit spell requirement. Whether a closed container blocks the magic depends on whether it provides total cover, so resolve that with the DM.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A20" s="37" t="str">
-        <x:v>What it does not do</x:v>
-      </x:c>
-      <x:c r="B20" s="38" t="str">
-        <x:v>It does not affect magical food or drink, cure a poisoned or diseased creature, create food or water, detect poison, or make every non-food substance edible. It only removes poison and disease from qualifying food and drink. Other contamination, spoilage, and whether something counts as food or drink may require a DM ruling.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A21" s="35" t="str">
-        <x:v>Duration</x:v>
-      </x:c>
-      <x:c r="B21" s="36" t="str">
-        <x:v>The purification happens immediately. You do not maintain it, and dispelling magic afterward does not undo an instantaneous purification. The food or drink can be contaminated again later; it gains no lasting protective ward.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A22" s="37" t="str">
-        <x:v>Ritual restriction</x:v>
-      </x:c>
-      <x:c r="B22" s="38" t="str">
-        <x:v>The spell has a ritual tag, but the 2014 Paladin class does not grant ritual casting. Bob must prepare it and spend 1 spell slot for his normal 1-action cast. Only a separate feature that actually permits this spell as a ritual would allow a slot-free casting with 10 additional minutes.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A23" s="35" t="str">
+      <x:c r="A19" s="41" t="str">
         <x:v>Higher slots</x:v>
       </x:c>
-      <x:c r="B23" s="36" t="str">
-        <x:v>You may spend a higher-level slot if available, but this spell lists no increase in radius, range, or effect. Bob has only 1st-level slots at level 2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="37" t="str">
+      <x:c r="B19" s="42" t="str">
+        <x:v>One additional willing creature per slot level above 1st; touch each target when casting. This does not increase temporary HP per target or duration. Bob cannot upcast at Paladin level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="43" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="B24" s="38" t="str">
-        <x:v>https://www.dnd5eapi.co/api/2014/spells/purify-food-and-drink</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="33" t="str">
-        <x:v>Bless</x:v>
-      </x:c>
-      <x:c r="B25" s="33" t="str">
-        <x:v>Level 1; 1 action; 30 ft; Up to 1 minute; concentration</x:v>
+      <x:c r="B20" s="44" t="str">
+        <x:v>https://dnd5e.wikidot.com/spell:heroism</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="40" t="str">
+        <x:v>Thunderous Smite</x:v>
+      </x:c>
+      <x:c r="B21" s="40" t="str">
+        <x:v>Level 1; 1 bonus action; Self; Up to 1 minute; concentration</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A22" s="43" t="str">
+        <x:v>School &amp; components</x:v>
+      </x:c>
+      <x:c r="B22" s="44" t="str">
+        <x:v>1st-level evocation, 2014 Player’s Handbook. Verbal (V) only: you must speak; no free-hand gesture, material, or holy symbol is required. Not a ritual. Concentration up to 1 minute, normally 10 rounds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A23" s="41" t="str">
+        <x:v>Cast before attacking</x:v>
+      </x:c>
+      <x:c r="B23" s="42" t="str">
+        <x:v>Spend a bonus action and a spell slot before the hit you want to empower. You may then take the Attack action on that turn. This is the 2014 spell, not a spell cast as a reaction to hitting. You cannot cast Cure Wounds or Heroism on the same turn as this bonus-action spell; see shared casting rules.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A24" s="43" t="str">
+        <x:v>Trigger &amp; damage</x:v>
+      </x:c>
+      <x:c r="B24" s="44" t="str">
+        <x:v>Your first melee weapon attack that hits during the duration deals an extra 2d6 thunder damage. Roll the normal weapon attack, not your spell attack modifier. A miss does not trigger the extra damage; you can try again while concentration and duration last. Only the first qualifying hit benefits; subsequent hits need a new casting. After the hit there is no remaining benefit to maintain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A25" s="41" t="str">
+        <x:v>Push &amp; prone</x:v>
+      </x:c>
+      <x:c r="B25" s="42" t="str">
+        <x:v>If that hit targets a creature, it also makes a Strength saving throw against your spell save DC. Failure pushes it 10 ft away from you and knocks it prone. Success prevents both push and prone but does not cancel the extra thunder damage. The spell states no size limit; creature immunities or specific traits can still matter. An object does not make this creature-only save.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A26" s="37" t="str">
-        <x:v>School &amp; components</x:v>
-      </x:c>
-      <x:c r="B26" s="38" t="str">
-        <x:v>1st-level enchantment. Verbal, somatic, and material (V, S, M): a sprinkling of holy water. This spell states no component cost and does not say the material is consumed. A component pouch or your Paladin holy-symbol focus can replace that material. You still need speech and the required hand access; the hand used for the material or focus can also perform the somatic gesture. Not a ritual.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A27" s="35" t="str">
-        <x:v>Targets</x:v>
-      </x:c>
-      <x:c r="B27" s="36" t="str">
-        <x:v>Choose up to three creatures within 30 ft, including yourself if desired. You need a clear path to each target; total cover blocks targeting. The spell does not explicitly require sight or a willing target, and lists no creature-type exclusion. No saving throw or spell attack is required.</x:v>
+      <x:c r="A26" s="43" t="str">
+        <x:v>Weapon restrictions</x:v>
+      </x:c>
+      <x:c r="B26" s="44" t="str">
+        <x:v>A javelin used in melee qualifies; a thrown javelin or other ranged weapon attack does not trigger the spell. Bob’s lost greatsword is unavailable. Normal reach and attack restrictions still apply. The extra damage is thunder, not radiant, and damage resistance or immunity applies normally.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A27" s="41" t="str">
+        <x:v>Noise &amp; positioning</x:v>
+      </x:c>
+      <x:c r="B27" s="42" t="str">
+        <x:v>The empowered hit makes thunder audible within 300 ft; this can alert others and is not area damage. Forced movement from the push does not itself provoke opportunity attacks. After the push, check distance before using prone’s attack-roll effects: attacks from within 5 ft have advantage, farther attacks have disadvantage. A prone creature has disadvantage on its attacks and normally spends half its speed to stand.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A28" s="37" t="str">
-        <x:v>Benefit</x:v>
-      </x:c>
-      <x:c r="B28" s="38" t="str">
-        <x:v>Until the spell ends, each target can roll 1d4 and add it whenever it makes an attack roll or saving throw. Roll the bonus for each eligible roll; it is not used up after one roll. This includes death saving throws. It does not add to damage, AC, ability checks, skill checks, or initiative.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A29" s="35" t="str">
-        <x:v>Duration &amp; range</x:v>
-      </x:c>
-      <x:c r="B29" s="36" t="str">
-        <x:v>Concentration, up to 1 minute (normally 10 combat rounds). Once cast, targets can move beyond 30 ft without losing the spell. You cannot transfer the benefit to new targets without casting again. Multiple Bless castings on one target do not stack into extra d4s.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A30" s="37" t="str">
-        <x:v>Concentration limits</x:v>
-      </x:c>
-      <x:c r="B30" s="38" t="str">
-        <x:v>You may concentrate on only one spell at a time. Casting another concentration spell, being incapacitated, or dying ends Bless. You may end it voluntarily at any time without an action. Ordinary movement and attacks do not break it. Casting Command or Purify Food and Drink does not itself break Bless because neither requires concentration.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A31" s="35" t="str">
-        <x:v>Damage checks</x:v>
-      </x:c>
-      <x:c r="B31" s="36" t="str">
-        <x:v>Each separate source of damage requires your Constitution saving throw: DC 10 or half the damage actually taken, whichever is higher (round fractions down). Failure ends Bless for every target. Your Constitution save bonus is shown in the casting reference below. If you included yourself in Bless, its d4 applies to this save while the spell is still active. The DM can also call for a DC 10 check for severe environmental disruption.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A32" s="37" t="str">
+      <x:c r="A28" s="43" t="str">
+        <x:v>Concentration &amp; expiry</x:v>
+      </x:c>
+      <x:c r="B28" s="44" t="str">
+        <x:v>Casting this ends your Heroism or any other concentration spell. Casting another concentration spell, a failed concentration check, incapacitation, death, or voluntary ending stops this spell. If it expires or ends before a qualifying hit, the slot is still spent and there is no bonus damage. See shared rules for damage checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A29" s="41" t="str">
+        <x:v>Other smites &amp; critical hits</x:v>
+      </x:c>
+      <x:c r="B29" s="42" t="str">
+        <x:v>You can add the separate Divine Smite class feature to the same melee hit if you spend another spell slot. It is not another spell cast, so the bonus-action casting restriction does not forbid it. You need two available slots to fund both effects. On a critical hit, double the weapon’s damage dice and this spell’s extra dice (4d6 thunder); do not double flat modifiers. Great Weapon Fighting does not reroll the spell’s thunder dice.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="43" t="str">
         <x:v>Higher slots</x:v>
       </x:c>
-      <x:c r="B32" s="38" t="str">
-        <x:v>Add one target for each slot level above 1st: four targets with a 2nd-level slot, five with a 3rd-level slot, and so on. Each starts within 30 ft of you; there is no additional distance-between-targets restriction. Higher slots do not increase the d4 or duration. Bob cannot upcast at level 2.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="35" t="str">
+      <x:c r="B30" s="44" t="str">
+        <x:v>No increased damage, distance, or target count is listed for higher slots. Bob has only 1st-level slots at Paladin level 2.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="41" t="str">
         <x:v>Source</x:v>
       </x:c>
-      <x:c r="B33" s="36" t="str">
-        <x:v>https://www.dnd5eapi.co/api/2014/spells/bless</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="33" t="str">
+      <x:c r="B31" s="42" t="str">
+        <x:v>https://dnd5e.wikidot.com/spell:thunderous-smite</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="40" t="str">
         <x:v>Shared casting rules</x:v>
       </x:c>
-      <x:c r="B34" s="33" t="str">
+      <x:c r="B32" s="40" t="str">
         <x:v>Applies to Bob’s 2014 Paladin spellcasting</x:v>
       </x:c>
     </x:row>
+    <x:row r="33" ht="66" hidden="0" customHeight="1">
+      <x:c r="A33" s="41" t="str">
+        <x:v>Preparation</x:v>
+      </x:c>
+      <x:c r="B33" s="42" t="str">
+        <x:v>Prepare Paladin spells of levels for which you have slots. The limit is Charisma modifier + half Paladin level rounded down, minimum 1 once spellcasting starts at level 2. Change the list after a long rest, with at least 1 minute of prayer and meditation per spell level for every spell on the new list. These three 1st-level selections require at least 3 minutes if all three are allowed. Bob currently has a limit of 2 because of the temporary Charisma penalty; all three requested choices are recorded pending bathing or a DM ruling. No completed rest or bath has been recorded for this selection. Casting a spell does not unprepare it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A34" s="43" t="str">
+        <x:v>Slots &amp; recovery</x:v>
+      </x:c>
+      <x:c r="B34" s="44" t="str">
+        <x:v>Each cast of Cure Wounds, Heroism, or Thunderous Smite uses one slot of 1st level or higher. They and Divine Smite share Bob’s two 1st-level slots at level 2: two uses total in any combination after full recovery. See the live slot counter for remaining uses. A long rest restores spent slots; a short rest does not. A miss, successful save, early ending, or unused effect does not refund a spent slot. None of these three spells can be cast as a ritual.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="35" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A35" s="35" t="str">
-        <x:v>Preparation</x:v>
-      </x:c>
-      <x:c r="B35" s="36" t="str">
-        <x:v>Your prepared-spell limit is Charisma modifier + half Paladin level rounded down, minimum 1 once spellcasting starts at level 2. Choose Paladin spells of levels for which you have slots. You can change the list after a long rest, with at least 1 minute of prayer and meditation per spell level for every spell on the new list. Bob's three 1st-level spells take at least 3 minutes to prepare. Casting a spell does not unprepare it.</x:v>
+      <x:c r="A35" s="41" t="str">
+        <x:v>Actions &amp; armor</x:v>
+      </x:c>
+      <x:c r="B35" s="42" t="str">
+        <x:v>Cure Wounds and Heroism take 1 action; Thunderous Smite takes 1 bonus action before the qualifying hit. Under 2014 rules, casting any bonus-action spell on your turn limits other spells that turn to a cantrip with a casting time of 1 action. Thus Thunderous Smite and either other selected spell cannot be cast on the same turn. Taking the Attack action is allowed. Bob can cast in his chain mail because he is proficient; armor you lack proficiency in prevents spellcasting.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A36" s="37" t="str">
-        <x:v>Slots &amp; recovery</x:v>
-      </x:c>
-      <x:c r="B36" s="38" t="str">
-        <x:v>Every normal cast uses one slot of the spell's level or higher. Command, Purify Food and Drink, Bless, and Divine Smite share Bob's two 1st-level slots at level 2. Two uses total, in any combination. A long rest restores spent slots; a short rest does not. A target succeeding on its save or a spell ending early does not refund a spent slot.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A37" s="35" t="str">
-        <x:v>Actions &amp; armor</x:v>
-      </x:c>
-      <x:c r="B37" s="36" t="str">
-        <x:v>All three recorded spells take 1 action, so they normally use the action you could otherwise use to attack. Under 2014 rules, casting any bonus-action spell on your turn limits other spells that turn to a cantrip with a casting time of 1 action. This is not a blanket one-spell-per-turn rule. Bob can cast in his chain mail because he is proficient with it; wearing armor you lack proficiency in prevents spellcasting.</x:v>
+      <x:c r="A36" s="43" t="str">
+        <x:v>Speech &amp; hands</x:v>
+      </x:c>
+      <x:c r="B36" s="44" t="str">
+        <x:v>All three spells need verbal components, so being gagged or inside magical silence prevents casting. Cure Wounds and Heroism also need somatic gestures with a free hand. A weapon-holding hand cannot freely make these gestures without a feature permitting it. Thunderous Smite requires only speech. A focus replaces eligible material components only; it does not replace speech or gestures.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A37" s="41" t="str">
+        <x:v>Holy symbol</x:v>
+      </x:c>
+      <x:c r="B37" s="42" t="str">
+        <x:v>A Paladin may use a holy symbol as a focus by holding it, wearing it visibly, or bearing it on a shield. Bob’s symbol form is unconfirmed. None of these three spells requires material components, so the symbol is not needed and does not remove the free-hand requirement for Cure Wounds or Heroism. For other spells, separately specified costly or consumed materials still must be supplied.</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A38" s="37" t="str">
-        <x:v>Speech &amp; hands</x:v>
-      </x:c>
-      <x:c r="B38" s="38" t="str">
-        <x:v>All three spells need verbal components, so being gagged or inside magical silence prevents their casting. Purify and Bless also require somatic gestures. A hand holding a weapon cannot freely perform those gestures unless another rule permits it. A focus can replace only eligible material components, not verbal or somatic requirements. Purify has no material component, so merely holding a focus does not remove its free-hand requirement.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A39" s="35" t="str">
-        <x:v>Holy symbol</x:v>
-      </x:c>
-      <x:c r="B39" s="36" t="str">
-        <x:v>A Paladin can use a holy symbol as a spellcasting focus, holding it, wearing it visibly, or bearing it on a shield. Bob has a holy symbol recorded, but its form is unconfirmed. Bless's material can be replaced by this focus; a separately specified costly or consumed material would still have to be supplied. Neither Command nor Purify needs a material component.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A40" s="37" t="str">
+      <x:c r="A38" s="43" t="str">
         <x:v>Choosing targets</x:v>
       </x:c>
-      <x:c r="B40" s="38" t="str">
-        <x:v>At casting, obey the spell's range, target type, sight requirement if stated, and clear-path rule. Total cover blocks targeting, even when a target is visible through an obstruction. Effects normally continue beyond casting range unless the spell says otherwise. Areas spread from their origin in unblocked straight lines; total cover excludes the blocked part.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A41" s="35" t="str">
+      <x:c r="B38" s="44" t="str">
+        <x:v>Obey each spell’s range, target type, willingness and any stated sight requirement. Total cover blocks targeting even if the target can be seen through an obstruction. Cure Wounds and Heroism require actual touch at casting, not a ranged spell attack; neither explicitly requires sight. Heroism requires willingness. Effects normally continue beyond casting range unless stated otherwise. Areas spread along unblocked lines from their origin; total cover excludes blocked parts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="66" hidden="0" customHeight="1">
+      <x:c r="A39" s="41" t="str">
         <x:v>Concentration</x:v>
       </x:c>
-      <x:c r="B41" s="36" t="str">
-        <x:v>Only Bless among Bob's three spells needs it. Keep one concentration effect at a time. Damage checks use Constitution, not Charisma and not your spell save DC. Each damage source has its own check, DC max(10, half damage taken rounded down). Incapacitation, death, a new concentration spell, voluntary ending, or a failed required check ends it.</x:v>
+      <x:c r="B39" s="42" t="str">
+        <x:v>Heroism and Thunderous Smite both require it; you cannot maintain both. Casting either ends the other immediately. Cure Wounds does not require concentration. Each separate source of damage to Bob requires a Constitution saving throw, DC 10 or half the damage taken rounded down, whichever is higher. Damage absorbed by temporary HP counts. Failure, incapacitation, death, or starting another concentration spell ends concentration. You can end it voluntarily without an action. The DM can require a DC 10 check for severe environmental disruption. Normal movement and attacks do not break it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="66" hidden="0" customHeight="1">
+      <x:c r="A40" s="43" t="str">
+        <x:v>Saves versus attacks</x:v>
+      </x:c>
+      <x:c r="B40" s="44" t="str">
+        <x:v>Spell save DC is 8 + proficiency bonus + Charisma modifier. Spell attack modifier is proficiency bonus + Charisma modifier. Cure Wounds and Heroism use neither a saving throw nor an attack roll. Thunderous Smite uses a normal melee weapon attack; its creature target then rolls Strength against your spell DC for push and prone only. Divine Smite is a class feature triggered by a melee weapon hit. A melee javelin qualifies for either smite; a thrown javelin does not. When an enemy casts at Bob, roll the saving throw that enemy spell requires against the enemy’s DC, not Bob’s spell save DC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A41" s="41" t="str">
+        <x:v>Rules sources</x:v>
+      </x:c>
+      <x:c r="B41" s="42" t="str">
+        <x:v>Rules and practical notes paraphrased from 2014 fifth edition. Cure Wounds, Heroism, and general casting: SRD 5.1 by Wizards of the Coast LLC, licensed under CC BY 4.0, https://creativecommons.org/licenses/by/4.0/ . SRD: https://media.wizards.com/2023/downloads/dnd/SRD_CC_v5.1.pdf . Casting: https://www.dnd5eapi.co/api/2014/rule-sections/casting-a-spell . Paladin: https://www.dnd5eapi.co/api/2014/classes/paladin . Thunderous Smite: 2014 Player’s Handbook, reference https://dnd5e.wikidot.com/spell:thunderous-smite . Heroism higher slots: https://dnd5e.wikidot.com/spell:heroism . Specific traits and DM rulings can change interactions.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A42" s="37" t="str">
-        <x:v>Saves versus attacks</x:v>
-      </x:c>
-      <x:c r="B42" s="38" t="str">
-        <x:v>Command makes its target roll Wisdom against your spell save DC. Bless and Purify require neither a save nor a spell attack roll. Your spell attack modifier therefore is not rolled for any of these three spells. Divine Smite is a class feature triggered by a melee weapon hit, not a separate spell attack; a thrown javelin does not qualify, but a melee javelin hit can.</x:v>
-      </x:c>
+      <x:c r="A42" s="28"/>
+      <x:c r="B42" s="28"/>
     </x:row>
     <x:row r="43" ht="66" hidden="0" customHeight="1">
-      <x:c r="A43" s="35" t="str">
-        <x:v>Rules sources</x:v>
-      </x:c>
-      <x:c r="B43" s="36" t="str">
-        <x:v>2014 SRD 5.1 spell and spellcasting rules, paraphrased with practical notes. Sources: https://www.dnd5eapi.co/api/2014/rule-sections/casting-a-spell ; https://www.dnd5eapi.co/api/2014/rule-sections/what-is-a-spell ; https://www.dnd5eapi.co/api/2014/classes/paladin . Source text: https://media.wizards.com/2023/downloads/dnd/SRD_CC_v5.1.pdf . SRD 5.1 by Wizards of the Coast LLC is licensed under CC BY 4.0: https://creativecommons.org/licenses/by/4.0/ . Specific creature traits and your DM's rulings can change an interaction.</x:v>
-      </x:c>
+      <x:c r="A43" s="28"/>
+      <x:c r="B43" s="28"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="28"/>
@@ -3792,6 +3818,54 @@
     <x:row r="48">
       <x:c r="A48" s="28"/>
       <x:c r="B48" s="28"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="28"/>
+      <x:c r="B49" s="28"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="28"/>
+      <x:c r="B50" s="28"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="28"/>
+      <x:c r="B51" s="28"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="28"/>
+      <x:c r="B52" s="28"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="28"/>
+      <x:c r="B53" s="28"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="28"/>
+      <x:c r="B54" s="28"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="28"/>
+      <x:c r="B55" s="28"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="28"/>
+      <x:c r="B56" s="28"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="28"/>
+      <x:c r="B57" s="28"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="28"/>
+      <x:c r="B58" s="28"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="28"/>
+      <x:c r="B59" s="28"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="28"/>
+      <x:c r="B60" s="28"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Update Bob after long rest with greathammer and height
</commit_message>
<xml_diff>
--- a/public/dnd/Bob_the_Paladin.xlsx
+++ b/public/dnd/Bob_the_Paladin.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R76a66233b52d44c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="Rcceadbd1eb0f4cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="Rb457a6852da84252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R52359aa56af64ce9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R8bbb0fb33a87437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Character" sheetId="1" r:id="R3484ba36be3945ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spellbook" sheetId="2" r:id="R3a2b70d04e954b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="3" r:id="R89999dcd61664a49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journal" sheetId="4" r:id="R16f916ddb7a8439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spell details" sheetId="5" r:id="R485b7c512f3b46df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,7 +320,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8cbf8847dd894e5f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rce3acfc0410e4f30"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -950,7 +950,7 @@
         <x:v>Current HP</x:v>
       </x:c>
       <x:c r="H22" s="9" t="n">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="I22" s="5"/>
       <x:c r="J22" s="5"/>
@@ -961,18 +961,18 @@
         <x:v>CHA</x:v>
       </x:c>
       <x:c r="B23" s="9" t="n">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C23" s="11" t="n">
         <x:f>INT((B23-10)/2)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E23" s="11" t="n">
         <x:f>C23+IF(D23="Yes",$E$10,0)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F23" s="5"/>
       <x:c r="G23" s="5" t="str">
@@ -1164,7 +1164,7 @@
       </x:c>
       <x:c r="D31" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B31,$A$18:$A$23,0))+IF(C31="Yes",$E$10,0)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E31" s="5"/>
       <x:c r="F31" s="5"/>
@@ -1240,7 +1240,7 @@
       </x:c>
       <x:c r="D34" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B34,$A$18:$A$23,0))+IF(C34="Yes",$E$10,0)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E34" s="5"/>
       <x:c r="F34" s="5"/>
@@ -1390,7 +1390,7 @@
       </x:c>
       <x:c r="D39" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B39,$A$18:$A$23,0))+IF(C39="Yes",$E$10,0)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E39" s="5"/>
       <x:c r="F39" s="5"/>
@@ -1412,7 +1412,7 @@
       </x:c>
       <x:c r="D40" s="11" t="n">
         <x:f>INDEX($C$18:$C$23,MATCH(B40,$A$18:$A$23,0))+IF(C40="Yes",$E$10,0)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E40" s="5"/>
       <x:c r="F40" s="5"/>
@@ -1707,7 +1707,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e4a86900c94d28"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8eeb585b3a624837"/>
 </x:worksheet>
 </file>
 
@@ -1799,7 +1799,7 @@
       </x:c>
       <x:c r="G6" s="10" t="n">
         <x:f>IF(Character!B10&lt;2,"Not unlocked",8+Character!E10+Character!C23)</x:f>
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H6" s="5"/>
     </x:row>
@@ -1812,11 +1812,11 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="9" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="10" t="n">
         <x:f>B7-C7</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E7" s="5"/>
       <x:c r="F7" s="5" t="str">
@@ -1824,7 +1824,7 @@
       </x:c>
       <x:c r="G7" s="11" t="n">
         <x:f>IF(Character!B10&lt;2,"Not unlocked",Character!E10+Character!C23)</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H7" s="5"/>
     </x:row>
@@ -1849,7 +1849,7 @@
       </x:c>
       <x:c r="G8" s="10" t="n">
         <x:f>IF(Character!B10&lt;2,0,MAX(1,Character!C23+INT(Character!B10/2)))</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H8" s="5"/>
     </x:row>
@@ -1899,7 +1899,7 @@
       </x:c>
       <x:c r="G10" s="10" t="str">
         <x:f>IF(G9&gt;G8,"Over limit","Within limit")</x:f>
-        <x:v>Over limit</x:v>
+        <x:v>Within limit</x:v>
       </x:c>
       <x:c r="H10" s="5"/>
     </x:row>
@@ -3137,14 +3137,23 @@
         <x:v>Gaming set proficiency</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="38" customHeight="1">
-      <x:c r="A17" s="18"/>
-      <x:c r="B17" s="18"/>
-      <x:c r="C17" s="22"/>
-      <x:c r="D17" s="23" t="str">
-        <x:f>IF(A17="","",B17*C17)</x:f>
-      </x:c>
-      <x:c r="E17" s="18"/>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" s="18" t="str">
+        <x:v>Greathammer</x:v>
+      </x:c>
+      <x:c r="B17" s="18" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D17" s="23" t="n">
+        <x:f>B17*C17</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="str">
+        <x:v>Two-handed; 1d8 bludgeoning. Newly acquired. Weight and any additional properties not recorded.</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
       <x:c r="A18" s="18"/>
@@ -3347,7 +3356,7 @@
       <x:c r="A12" s="5"/>
       <x:c r="B12" s="5"/>
     </x:row>
-    <x:row r="13" ht="570" customHeight="1">
+    <x:row r="13" ht="900" customHeight="1">
       <x:c r="A13" s="25" t="str">
         <x:v>Adventure notes</x:v>
       </x:c>
@@ -3361,7 +3370,13 @@
 Encounter update — September 13, 2026 (Kai): initiative 19 (rolled 18 + 1). Cast Bless on the druid, Cat, and Taric, spending one 1st-level spell slot; 1 of 2 slots remains. Bob maintains concentration, up to 1 minute (10 rounds), unless it ends earlier. These three targets add 1d4 to attack rolls and saving throws; Bob is not a target. Pulled right arm; Kai confirmed no HP damage, so HP remains 15/20. No mechanical penalty was specified; any penalty needs a DM ruling.
 Falling rocks — September 13, 2026 (Kai): took 2 damage, reducing HP from 15/20 to 13/20. Kai clarified that Bless had already ended. The druid, Cat, and Taric no longer receive its bonus; no concentration save was needed for this damage. One 1st-level spell slot remains.
 Covered in blood and guts — September 13, 2026 (Kai): -2 Charisma until Bob takes a bath. Applied to the score: 14 to 12, modifier +1. Base score 14 is retained here for restoration after bathing. HP stays 13/20 and one 1st-level spell slot remains. The three prepared spells are retained; the reduced preparation limit of 2 needs a DM ruling. Divine Sense counters are unchanged pending the DM ruling on how this temporary effect affects its pool.
-Spell selection — September 14, 2026 (Kai): Cure Wounds, Heroism, and Thunderous Smite replace Command, Purify Food and Drink, and Bless in the recorded list. This records the requested next preparation; no completed long rest, bath, healing, casting, or resource recovery is assumed. HP remains 13/20; one 1st-level slot remains. The current preparation limit is 2 with Charisma 12; all three choices are retained pending bathing (restoring Charisma 14 and limit 3) or the DM’s ruling. Heroism and Thunderous Smite cannot be concentrated on together.</x:v>
+Spell selection — September 14, 2026 (Kai): Cure Wounds, Heroism, and Thunderous Smite replace Command, Purify Food and Drink, and Bless in the recorded list. This records the requested next preparation; no completed long rest, bath, healing, casting, or resource recovery is assumed. HP remains 13/20; one 1st-level slot remains. The current preparation limit is 2 with Charisma 12; all three choices are retained pending bathing (restoring Charisma 14 and limit 3) or the DM’s ruling. Heroism and Thunderous Smite cannot be concentrated on together.
+Bath — September 20, 2026 (Kai): took a bath and removed the blood-and-guts debuff. Charisma restored from 12 to 14 (+2 modifier). Spell save DC 12; spell attack +4; Charisma save +4; preparation limit 3. All three recorded selections now fit the limit. HP remains 13/20 and one 1st-level spell slot remains. No long rest, healing, casting, or resource recovery recorded.
+Navigation — September 20, 2026 (Kai): Compass Rose → go north to the ship.
+Ship clues and agreement — September 20, 2026 (Kai): “mermaid like creature holding the compass ship with compass”. Anything we find on that ship is ours to keep.
+New weapon — September 20, 2026 (Kai): acquired one Greathammer, dealing 1d8 bludgeoning. Weight and weapon properties not specified.
+Weapon clarification — September 20, 2026 (Kai): the Greathammer requires two hands. Damage remains 1d8 bludgeoning.
+Long rest — September 20, 2026 (Kai): completed a long rest. HP restored to 20/20; both 1st-level spell slots available; hit dice available 2d10; Fire Breath 1/1, Divine Sense 3/3, and Lay on Hands 10/10. Charisma remains 14 after the bath. The three recorded spell selections fit the preparation limit; their prayer and meditation takes at least 3 minutes.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
@@ -3402,10 +3417,10 @@
     </x:row>
     <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="17" t="str">
-        <x:v>Covered in blood and guts</x:v>
+        <x:v>Height</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
-        <x:v>Temporary -2 Charisma score until Bob takes a bath: base 14, current 12 (+1 modifier). Restore Charisma to 14 after the bath. Spell save DC 11; spell attack +3; Charisma save +3. Current prepared-spell limit is 2; all 3 selected spells are recorded pending the DM ruling on this temporary penalty.</x:v>
+        <x:v>196 cm (approximately 6 ft 5 in). Confirmed by Kai.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
@@ -3475,7 +3490,7 @@
     </x:row>
     <x:row r="2" ht="44" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>3 selections recorded; current preparation limit 2 (DM check). Two shared 1st-level slots; 1 remains. Heroism and Thunderous Smite cannot be maintained together. No rest or bath assumed.</x:v>
+        <x:v>Long rest completed. HP 20/20; both 1st-level slots available. Charisma 14; preparation limit 3 for the three recorded selections. Heroism and Thunderous Smite cannot be maintained together.</x:v>
       </x:c>
       <x:c r="B2" s="28"/>
     </x:row>
@@ -3724,7 +3739,7 @@
         <x:v>Preparation</x:v>
       </x:c>
       <x:c r="B33" s="42" t="str">
-        <x:v>Prepare Paladin spells of levels for which you have slots. The limit is Charisma modifier + half Paladin level rounded down, minimum 1 once spellcasting starts at level 2. Change the list after a long rest, with at least 1 minute of prayer and meditation per spell level for every spell on the new list. These three 1st-level selections require at least 3 minutes if all three are allowed. Bob currently has a limit of 2 because of the temporary Charisma penalty; all three requested choices are recorded pending bathing or a DM ruling. No completed rest or bath has been recorded for this selection. Casting a spell does not unprepare it.</x:v>
+        <x:v>Prepare Paladin spells of levels for which you have slots. The limit is Charisma modifier + half Paladin level rounded down, minimum 1 once spellcasting starts at level 2. Change the list after a long rest, with at least 1 minute of prayer and meditation per spell level for every spell on the new list. These three 1st-level selections require at least 3 minutes of preparation. Bob has taken a bath and removed the temporary Charisma penalty: Charisma 14 gives a preparation limit of 3, so all three recorded choices fit. Kai confirmed a completed long rest on September 20, 2026. The three recorded spell selections fit the preparation limit of 3; preparing them requires at least 3 minutes of prayer and meditation. Casting a spell does not unprepare it.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="52.79999923706055" hidden="0" customHeight="1">

</xml_diff>